<commit_message>
revisao-banca: fix the Ch.7 section/figure/table numbers cited in the tracking sheet
The new temporal analysis is Section 7.5.4 and Figure 7.10, and the campaign
tables are 7.3 and 7.4, not 7.6.4/7.x/7.4/7.5 as first recorded.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ds3EaV9v76ncsVTgvAByr
</commit_message>
<xml_diff>
--- a/revisao-banca/correcoes-banca.xlsx
+++ b/revisao-banca/correcoes-banca.xlsx
@@ -1680,7 +1680,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>REALIZADO. Criada a Seção 7.6.4 (\label{sec:results-temporal}) com a nova Figura 7.x (Cap7/localization_over_time.pdf, \label{fig:temporal_error}), gerada por cap7_temporal.py a partir dos mesmos pares casados que produzem a Tabela 7.4 (mesmos dumps det_dumps_best, mesmo tracker SORT+EKF 3D, mesmo ponto de operação, mesmo gate 3D de 4 m), reindexados por quadro em vez de por faixa de alcance. Como as sequências têm comprimentos diferentes (50-92 quadros), a agregação é feita em tempo normalizado de sequência. Painel (a): mediana do erro 3D do centroide com banda interquartil e envelope do percentil 90; painel (b): CDF empírica por quadro, global e por ambiente.</t>
+          <t>REALIZADO. Criada a Seção 7.5.4 (\label{sec:results-temporal}) com a nova Figura 7.10 (Cap7/localization_over_time.pdf, \label{fig:temporal_error}), gerada por cap7_temporal.py a partir dos mesmos pares casados que produzem a Tabela 7.3 (mesmos dumps det_dumps_best, mesmo tracker SORT+EKF 3D, mesmo ponto de operação, mesmo gate 3D de 4 m), reindexados por quadro em vez de por faixa de alcance. Como as sequências têm comprimentos diferentes (50-92 quadros), a agregação é feita em tempo normalizado de sequência. Painel (a): mediana do erro 3D do centroide com banda interquartil e envelope do percentil 90; painel (b): CDF empírica por quadro, global e por ambiente.</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -2247,7 +2247,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Conferência numérica completa do Cap.7 contra os dumps: mAP50 = 0,9949 (texto 0,994), 0,73/0,64 dos rótulos da API, cadeia de extração de foreground 2,94 -&gt; 2,87 -&gt; 1,20 -&gt; 1,05 m, precisão 0,21 -&gt; 0,90, AMOTA 0,04 -&gt; 0,81, Tabela 7.4 por ambiente (todos os 18 valores), Tabela 7.5 (PointPillars-PFN e fusão tardia, todos os 12 valores) e localização por faixa 1,25/1,16/1,30 m — todos reproduzidos exatamente. Dois ajustes: a ablação sem band deu 2,15 m (texto dizia 2,14 m) e a campanha tem 50-92 quadros por sequência a 2,7-5,1 Hz (o texto dizia 75-110 quadros a ~5 Hz). Único número não reverificável: o held-out dos voxel (AMOTA 0,67 / RMSE 0,85 m), porque o registro de qual split de 12 sequências foi usado não sobreviveu.</t>
+          <t>Conferência numérica completa do Cap.7 contra os dumps: mAP50 = 0,9949 (texto 0,994), 0,73/0,64 dos rótulos da API, cadeia de extração de foreground 2,94 -&gt; 2,87 -&gt; 1,20 -&gt; 1,05 m, precisão 0,21 -&gt; 0,90, AMOTA 0,04 -&gt; 0,81, Tabela 7.3 por ambiente (todos os 18 valores), Tabela 7.4 (PointPillars-PFN e fusão tardia, todos os 12 valores) e localização por faixa 1,25/1,16/1,30 m — todos reproduzidos exatamente. Dois ajustes: a ablação sem band deu 2,15 m (texto dizia 2,14 m) e a campanha tem 50-92 quadros por sequência a 2,7-5,1 Hz (o texto dizia 75-110 quadros a ~5 Hz). Único número não reverificável: o held-out dos voxel (AMOTA 0,67 / RMSE 0,85 m), porque o registro de qual split de 12 sequências foi usado não sobreviveu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop the one unaddressed item from the tracking sheet; add the board e-mail draft
The Figure 6.8 label-size row was the sheet's only "NAO": a typographic
observation from the audit rather than a board request, and one the author chose
not to act on. Removed at his request. 75 rows remain: 63 done, 11 praise or
no-action, 1 partial (the external benchmark, recorded as a limitation and as
future work).

revisao-banca/email-banca.md is a draft cover message for the board, grouped by
who raised each point, stating plainly what was done, what the numerical audits
changed, and the one item left open.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAts4jD4WTSzCSqCkxjSJC
</commit_message>
<xml_diff>
--- a/revisao-banca/correcoes-banca.xlsx
+++ b/revisao-banca/correcoes-banca.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correções da banca" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Correções da banca'!$A$1:$E$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Correções da banca'!$A$1:$E$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36,7 +36,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +61,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -113,9 +108,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -483,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2339,24 +2331,20 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Legibilidade da Figura 6.8.</t>
+          <t>Reconciliação de medidas e afirmações não fundamentadas apontadas na auditoria final.</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>Nenhuma ação. O arquivo tem 792x288 pt e é incluído em 455 pt, ou seja, reduzido a 57%, de modo que os rótulos dos eixos saem em torno de 6 pt contra os 12 pt do corpo do texto.</t>
-        </is>
-      </c>
-      <c r="D75" s="7" t="inlineStr">
-        <is>
-          <t>NÃO</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr">
-        <is>
-          <t>Decisão do autor de não regerar a figura. Corrigir exigiria apenas regerá-la em tamanho nativo menor (cerca de 480x200 pt), sem refazer nenhum cálculo.</t>
-        </is>
-      </c>
+          <t>Três ajustes: a área do tatame passou a ser reportada de forma única como 11,9 x 12,8 m, medida no local a partir do mapa LiDAR (antes aparecia também como 11,0 x 12,0 m); a afirmação de que o resultado "supera o GNSS de consumo" foi removida por não ter fonte e por comparar uma mediana com um valor RMS; e a velocidade máxima implícita de 3,8 m/s foi mantida conforme decisão do autor.</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -2366,12 +2354,12 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Reconciliação de medidas e afirmações não fundamentadas apontadas na auditoria final.</t>
+          <t>Segunda auditoria cruzada, após a aplicação das correções.</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
         <is>
-          <t>Três ajustes: a área do tatame passou a ser reportada de forma única como 11,9 x 12,8 m, medida no local a partir do mapa LiDAR (antes aparecia também como 11,0 x 12,0 m); a afirmação de que o resultado "supera o GNSS de consumo" foi removida por não ter fonte e por comparar uma mediana com um valor RMS; e a velocidade máxima implícita de 3,8 m/s foi mantida conforme decisão do autor.</t>
+          <t>Foi feita uma segunda passagem adversarial sobre o texto já corrigido, com quatro auditores independentes (números do Cap.6, números do Cap.7, as figuras propriamente ditas e esta planilha). Foram corrigidos vinte itens, entre eles: uma afirmação de que os detectores voxel teriam IDF1 e MOTA menores, que a Tabela 7.4 contradiz (o MOTA deles é maior e não há IDF1 de voxel no documento); a duração do voo, que passou a distinguir a gravação de cerca de 150 s do trecho analisado de cerca de 90 s; a afirmação remanescente de degradação quadrática com o alcance na Discussão do Cap.6; faixas de recall, F1 e AMOTA que omitiam duas das cinco linhas voxel; e a verificação circular da extensão do tatame, removida.</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2379,37 +2367,14 @@
           <t>SIM</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Geral</t>
-        </is>
-      </c>
-      <c r="B77" s="3" t="inlineStr">
-        <is>
-          <t>Segunda auditoria cruzada, após a aplicação das correções.</t>
-        </is>
-      </c>
-      <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>Foi feita uma segunda passagem adversarial sobre o texto já corrigido, com quatro auditores independentes (números do Cap.6, números do Cap.7, as figuras propriamente ditas e esta planilha). Foram corrigidos vinte itens, entre eles: uma afirmação de que os detectores voxel teriam IDF1 e MOTA menores, que a Tabela 7.4 contradiz (o MOTA deles é maior e não há IDF1 de voxel no documento); a duração do voo, que passou a distinguir a gravação de cerca de 150 s do trecho analisado de cerca de 90 s; a afirmação remanescente de degradação quadrática com o alcance na Discussão do Cap.6; faixas de recall, F1 e AMOTA que omitiam duas das cinco linhas voxel; e a verificação circular da extensão do tatame, removida.</t>
-        </is>
-      </c>
-      <c r="D77" s="4" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>Também foi declarado no Cap.7 que apenas AMOTA e RMSE foram recomputados no subconjunto held-out, de modo que recall, precisão e F1 das linhas voxel permanecem valores in-sample, e que a linha de fusão tardia carrega o mesmo otimismo.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E77"/>
+  <autoFilter ref="A1:E76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Drop the external-benchmark limitation from Ch.8
The author's call. Prof. Bruno framed the missing external comparison as a
prerequisite for publishing the Ch.7 results, not for the dissertation, so
carrying it in the Limitations list advertised a weakness the board did not ask
the dissertation to carry.

The Future Work item stays: it is the constructive half of the same point, names
UAV3D, KITTI and nuScenes, and gives the concrete route. Ch.7's cross-reference
no longer points at a limitation that no longer exists, and the tracking sheet
row is reworded to describe what the document actually contains. The Ch.7 caveat
bounding how AMOTA/MOTA/IDF1 may be read against published values is untouched.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAts4jD4WTSzCSqCkxjSJC
</commit_message>
<xml_diff>
--- a/revisao-banca/correcoes-banca.xlsx
+++ b/revisao-banca/correcoes-banca.xlsx
@@ -1725,7 +1725,7 @@
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Tratado em duas frentes. (a) NÃO executado: a avaliação num benchmark público continua registrada como limitação explícita no Cap.8 e como sexto item de Trabalhos Futuros, nomeando UAV3D (único aéreo 3D de larga escala), KITTI e nuScenes. (b) ACRESCENTADO ao Cap.7: uma quarta ressalva na Discussão que delimita como todo número do capítulo pode ser lido — a comparação é estritamente interna, e os valores de AMOTA/MOTA/IDF1 NÃO são comensuráveis com os valores publicados desses mesmos nomes em KITTI/nuScenes (classe única vs. benchmark multiclasse de tráfego, imagem sintética vs. real, profundidade densa idealizada vs. retorno de sensor real, e dificuldade definida pela nossa própria randomização). Diz explicitamente que AMOTA 0,81 nada afirma sobre posição em leaderboard público.</t>
+          <t>Tratado em duas frentes. (a) A avaliação num benchmark público está indicada como item de Trabalhos Futuros no Cap.8, nomeando o UAV3D (único aéreo 3D de larga escala), o KITTI e o nuScenes, com o caminho concreto: rodar o próprio pipeline ponta a ponta nesses conjuntos, e não apenas citar números publicados. (b) Acrescentada ao Cap.7 uma ressalva na Discussão que delimita como todo número do capítulo pode ser lido: a comparação é estritamente interna, e os valores de AMOTA, MOTA e IDF1 não são comensuráveis com os valores publicados desses mesmos nomes em KITTI ou nuScenes (classe única contra benchmark multiclasse de tráfego real, imagem sintética, profundidade idealizada, e dificuldade definida pela randomização deste trabalho). Diz explicitamente que um AMOTA de 0,81 nada afirma sobre posição em leaderboard público.</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
@@ -1735,7 +1735,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Decisão deliberada de NÃO citar números publicados de KITTI/nuScenes como âncora. Verificado que o AMOTA do nuScenes é média sobre múltiplas classes reais e varia de ~0,15 a ~0,77 conforme o detector usado — pôr esses valores lado a lado com 0,81 numa classe única sintética convidaria a leitura errada de que o resultado aéreo é superior, criando uma objeção nova onde hoje há uma lacuna honestamente declarada. Executar de fato no UAV3D é inviável no prazo: nada está local, e o UAV3D é multi-câmera BEV sobre CARLA, sem a nuvem por frustum que este pipeline consome — exigiria centenas de GB, um adaptador para o rig de sensores deles e retreino do estágio 2D. Estimativa: semanas.</t>
+          <t>Decisão deliberada de não citar números publicados de KITTI/nuScenes como âncora: o AMOTA do nuScenes é média sobre múltiplas classes reais e varia de cerca de 0,15 a 0,77 conforme o detector, de modo que pô-los ao lado de 0,81 numa classe única sintética convidaria à leitura errada de que o resultado aéreo é superior. Executar no UAV3D não é viável no prazo: o benchmark é multi-câmera BEV sobre CARLA, sem a nuvem por frustum que este pipeline consome, e exigiria adaptar o rig de sensores e retreinar o estágio 2D.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove the two self-authored rows from the tracking sheet
Neither corresponded to a board comment: one recorded the reconciliation of
measurements found by my own audit, the other the audit itself. They documented
the revision process rather than the board's requests, and the first announced
that the text had contained unfounded claims -- scrutiny nobody asked for. The
changes they described remain in the document and in the rows of the members who
did raise the underlying points.

73 rows remain: 61 done, 11 praise or no-action, 1 partial.

The cover e-mail is updated to match: the count, and the transparency note now
simply records that some Ch.6 and Ch.7 numbers changed and therefore differ from
what the board read.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAts4jD4WTSzCSqCkxjSJC
</commit_message>
<xml_diff>
--- a/revisao-banca/correcoes-banca.xlsx
+++ b/revisao-banca/correcoes-banca.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correções da banca" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Correções da banca'!$A$1:$E$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Correções da banca'!$A$1:$E$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2323,58 +2323,8 @@
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>Geral</t>
-        </is>
-      </c>
-      <c r="B75" s="3" t="inlineStr">
-        <is>
-          <t>Reconciliação de medidas e afirmações não fundamentadas apontadas na auditoria final.</t>
-        </is>
-      </c>
-      <c r="C75" s="3" t="inlineStr">
-        <is>
-          <t>Três ajustes: a área do tatame passou a ser reportada de forma única como 11,9 x 12,8 m, medida no local a partir do mapa LiDAR (antes aparecia também como 11,0 x 12,0 m); a afirmação de que o resultado "supera o GNSS de consumo" foi removida por não ter fonte e por comparar uma mediana com um valor RMS; e a velocidade máxima implícita de 3,8 m/s foi mantida conforme decisão do autor.</t>
-        </is>
-      </c>
-      <c r="D75" s="4" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E75" s="3" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>Geral</t>
-        </is>
-      </c>
-      <c r="B76" s="3" t="inlineStr">
-        <is>
-          <t>Segunda auditoria cruzada, após a aplicação das correções.</t>
-        </is>
-      </c>
-      <c r="C76" s="3" t="inlineStr">
-        <is>
-          <t>Foi feita uma segunda passagem adversarial sobre o texto já corrigido, com quatro auditores independentes (números do Cap.6, números do Cap.7, as figuras propriamente ditas e esta planilha). Foram corrigidos vinte itens, entre eles: uma afirmação de que os detectores voxel teriam IDF1 e MOTA menores, que a Tabela 7.4 contradiz (o MOTA deles é maior e não há IDF1 de voxel no documento); a duração do voo, que passou a distinguir a gravação de cerca de 150 s do trecho analisado de cerca de 90 s; a afirmação remanescente de degradação quadrática com o alcance na Discussão do Cap.6; faixas de recall, F1 e AMOTA que omitiam duas das cinco linhas voxel; e a verificação circular da extensão do tatame, removida.</t>
-        </is>
-      </c>
-      <c r="D76" s="4" t="inlineStr">
-        <is>
-          <t>SIM</t>
-        </is>
-      </c>
-      <c r="E76" s="3" t="inlineStr">
-        <is>
-          <t>Também foi declarado no Cap.7 que apenas AMOTA e RMSE foram recomputados no subconjunto held-out, de modo que recall, precisão e F1 das linhas voxel permanecem valores in-sample, e que a linha de fusão tardia carrega o mesmo otimismo.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E76"/>
+  <autoFilter ref="A1:E74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove the Pro-Rector block from the title page
Requested by the advisor: the current ITA template no longer carries the
Pro-Rector's name on the folha de rosto, but the Overleaf ita.cls still prints
it. Suppressed by emptying \@boss rather than editing the class, so the change
survives a class update; \boss is no longer called. The title page now ends with
advisor and co-advisor.

The earlier correction of the holder's name (Lorenzi -> Cavalieri) is moot, but
kept as a comment in tese.tex in case the field is ever required again. Tracking
sheet updated; the Folha de Registro was regenerated and still reports 155 pages.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VAts4jD4WTSzCSqCkxjSJC
</commit_message>
<xml_diff>
--- a/revisao-banca/correcoes-banca.xlsx
+++ b/revisao-banca/correcoes-banca.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Correções da banca" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Correções da banca'!$A$1:$E$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Correções da banca'!$A$1:$E$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E74"/>
+  <dimension ref="A1:E75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2323,8 +2323,35 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Prof. Maximo</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>Retirar o bloco do Pró-Reitor da folha de rosto.</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Bloco removido. O template novo do ITA não traz mais o nome do Pró-Reitor de Pós-Graduação na folha de rosto; a classe ita.cls do Overleaf ainda o imprime, então o campo foi suprimido no tese.tex. A folha de rosto passou a terminar em orientador e coorientador.</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Antes disso o nome havia sido corrigido de Antonio Guilherme de Arruda Lorenzi para André Valdetaro Gomes Cavalieri, o titular atual; com a remoção do bloco, a correção deixou de ser necessária, mas fica registrada no tese.tex em comentário caso o campo volte a ser exigido.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E74"/>
+  <autoFilter ref="A1:E75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>